<commit_message>
Updated IO model files: GDP, Added value, Output, Gov and Household expenditures, and Percentage of household change
</commit_message>
<xml_diff>
--- a/InputData/fuels/BS/BAU Subsidies.xlsx
+++ b/InputData/fuels/BS/BAU Subsidies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/fuels/BS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D6B8620-F60E-2E48-B676-D20802CC40AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{037030F0-5568-BC41-A7EC-096C332B48ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="105">
   <si>
     <t>BS BAU Subsidy for Thermal Fuels per Energy Unit Produced ($/BTU)</t>
   </si>
@@ -357,9 +357,6 @@
   </si>
   <si>
     <t>$/BTU</t>
-  </si>
-  <si>
-    <t>Dollar/MWh</t>
   </si>
 </sst>
 </file>
@@ -2318,12 +2315,6 @@
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
       <c r="H12" s="9"/>
-      <c r="T12" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="U12" s="5">
-        <v>2.7276600000000001E-9</v>
-      </c>
     </row>
     <row r="13" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H13" s="9"/>
@@ -2528,12 +2519,8 @@
       <c r="P20" s="8"/>
       <c r="Q20" s="8"/>
       <c r="R20" s="8"/>
-      <c r="T20" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="U20" s="5">
-        <v>3.4024400000000003E-8</v>
-      </c>
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
       <c r="V20" s="8"/>
     </row>
     <row r="21" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2737,12 +2724,8 @@
       <c r="P28" s="8"/>
       <c r="Q28" s="8"/>
       <c r="R28" s="8"/>
-      <c r="T28" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="U28" s="5">
-        <v>1.3768E-8</v>
-      </c>
+      <c r="T28" s="8"/>
+      <c r="U28" s="8"/>
       <c r="V28" s="8"/>
     </row>
     <row r="29" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -41870,177 +41853,157 @@
         <v>0</v>
       </c>
       <c r="C2" s="14">
-        <v>0.39217710728623101</v>
+        <v>0</v>
       </c>
       <c r="D2" s="14">
-        <v>0.31989540904438946</v>
+        <v>0</v>
       </c>
       <c r="E2" s="14">
-        <v>0.33230210059378518</v>
+        <v>0</v>
       </c>
       <c r="F2" s="14">
-        <v>0.35053077387306397</v>
+        <v>0</v>
       </c>
       <c r="G2" s="14">
-        <v>0.41132451243803164</v>
+        <v>0</v>
       </c>
       <c r="H2" s="14">
-        <v>0.43166093130538014</v>
+        <v>0</v>
       </c>
       <c r="I2" s="14">
-        <v>0.44349134999614009</v>
+        <v>0</v>
       </c>
       <c r="J2" s="14">
-        <v>0.45846106071219805</v>
+        <v>0</v>
       </c>
       <c r="K2" s="14">
-        <v>0.4603413989714043</v>
+        <v>0</v>
       </c>
       <c r="L2" s="14">
-        <v>0.46268892759130964</v>
+        <v>0</v>
       </c>
       <c r="M2" s="14">
-        <v>0.47296355844160021</v>
+        <v>0</v>
       </c>
       <c r="N2" s="14">
-        <v>0.47743444223938519</v>
+        <v>0</v>
       </c>
       <c r="O2" s="14">
-        <v>0.4884105826167624</v>
+        <v>0</v>
       </c>
       <c r="P2" s="14">
-        <v>0.48455610506515023</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="14">
-        <v>0.50697090143679757</v>
+        <v>0</v>
       </c>
       <c r="R2" s="14">
-        <v>0.53367452355286327</v>
+        <v>0</v>
       </c>
       <c r="S2" s="14">
-        <v>0.5445107518984168</v>
+        <v>0</v>
       </c>
       <c r="T2" s="14">
-        <v>0.55611988748004071</v>
+        <v>0</v>
       </c>
       <c r="U2" s="14">
-        <v>0.55837210543599758</v>
+        <v>0</v>
       </c>
       <c r="V2" s="14">
-        <v>0.56005052626501151</v>
+        <v>0</v>
       </c>
       <c r="W2" s="14">
-        <v>0.56900861787829482</v>
+        <v>0</v>
       </c>
       <c r="X2" s="14">
-        <v>0.57020200392438491</v>
+        <v>0</v>
       </c>
       <c r="Y2" s="14">
-        <v>0.57602405402718537</v>
+        <v>0</v>
       </c>
       <c r="Z2" s="14">
-        <v>0.58542218669377366</v>
+        <v>0</v>
       </c>
       <c r="AA2" s="14">
-        <v>0.59267433657852298</v>
+        <v>0</v>
       </c>
       <c r="AB2" s="14">
-        <v>0.60620823184868677</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="14">
-        <v>0.61168648187983699</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="14">
-        <v>0.62309019997876425</v>
+        <v>0</v>
       </c>
       <c r="AE2" s="14">
-        <v>0.63517794046322185</v>
+        <v>0</v>
       </c>
       <c r="AF2" s="14">
-        <v>0.64052668305736016</v>
+        <v>0</v>
       </c>
       <c r="AG2" s="14">
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AH2" s="14">
-        <f t="shared" ref="D2:BA2" si="0">AG2</f>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AI2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AJ2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AK2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AL2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AM2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AN2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AO2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AP2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AQ2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AR2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AS2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AT2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AU2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AV2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AW2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AX2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AY2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="AZ2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
       <c r="BA2" s="14">
-        <f t="shared" si="0"/>
-        <v>0.63360124648119776</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>